<commit_message>
Final - PCB, Man. Files & BOM
</commit_message>
<xml_diff>
--- a/STMRocket - Manufacturing/STMRocket_BOM.xlsx
+++ b/STMRocket - Manufacturing/STMRocket_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sicoe\OneDrive\Desktop\Project - STMRocket\STMRocket - Manufacturing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A96F5BE-B923-4E6A-A4E6-C9BCE992BBDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15222379-3AAB-4B4B-AE32-8DA07B951792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="STMRocket BOM" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="143">
   <si>
     <t>xxxx xxxx xxxxx xxPCS BOM  (Sample Bill of Materials)</t>
   </si>
@@ -433,9 +433,6 @@
     <t>Amphenol</t>
   </si>
   <si>
-    <t>USB Micro-B</t>
-  </si>
-  <si>
     <t>XT30PW-M Horizontal Connector</t>
   </si>
   <si>
@@ -515,6 +512,15 @@
   </si>
   <si>
     <t>RES SMD 1.5K OHM 0.1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>USB Micro B</t>
+  </si>
+  <si>
+    <t>Screw Terminal</t>
+  </si>
+  <si>
+    <t>Pins</t>
   </si>
 </sst>
 </file>
@@ -707,56 +713,56 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1113,40 +1119,40 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:M38"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="16.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="9" style="1"/>
-    <col min="4" max="4" width="21.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="29.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="41.5546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.88671875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="35.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="41.5703125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="35.5703125" style="1" customWidth="1"/>
     <col min="10" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="19.5" customHeight="1">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="D2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="22"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
     </row>
     <row r="6" spans="1:12" ht="28.5" customHeight="1">
       <c r="A6" s="3" t="s">
@@ -1178,846 +1184,846 @@
       </c>
     </row>
     <row r="7" spans="1:12">
-      <c r="A7" s="10">
-        <v>1</v>
-      </c>
-      <c r="B7" s="11" t="s">
+      <c r="A7" s="8">
+        <v>1</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="10">
-        <v>1</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="C7" s="8">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I7" s="12"/>
+      <c r="H7" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="10"/>
     </row>
     <row r="8" spans="1:12">
-      <c r="A8" s="10">
+      <c r="A8" s="8">
         <v>2</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="10">
-        <v>1</v>
-      </c>
-      <c r="D8" s="9" t="s">
+      <c r="C8" s="8">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="H8" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" s="12"/>
+      <c r="H8" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="10"/>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="10">
+      <c r="A9" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="10">
-        <v>1</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="C9" s="8">
+        <v>1</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="H9" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I9" s="12"/>
+      <c r="H9" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="10">
+      <c r="A10" s="8">
         <v>4</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="10">
-        <v>1</v>
-      </c>
-      <c r="D10" s="9" t="s">
+      <c r="C10" s="8">
+        <v>1</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="H10" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="12"/>
+      <c r="H10" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="10"/>
     </row>
     <row r="11" spans="1:12">
-      <c r="A11" s="10">
+      <c r="A11" s="8">
         <v>5</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="10">
-        <v>1</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="C11" s="8">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="F11" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="H11" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I11" s="12"/>
+      <c r="H11" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" s="10"/>
     </row>
     <row r="12" spans="1:12">
-      <c r="A12" s="10">
+      <c r="A12" s="8">
         <v>6</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="10">
-        <v>1</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="C12" s="8">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="G12" s="17" t="s">
+      <c r="G12" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="H12" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I12" s="12"/>
+      <c r="H12" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I12" s="10"/>
     </row>
     <row r="13" spans="1:12">
-      <c r="A13" s="10">
+      <c r="A13" s="8">
         <v>7</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <v>2</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="G13" s="17" t="s">
+      <c r="G13" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="H13" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13" s="12"/>
-      <c r="L13" s="16"/>
+      <c r="H13" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="10"/>
+      <c r="L13" s="14"/>
     </row>
     <row r="14" spans="1:12">
-      <c r="A14" s="10">
+      <c r="A14" s="8">
         <v>8</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="10">
-        <v>1</v>
-      </c>
-      <c r="D14" s="9" t="s">
+      <c r="C14" s="8">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="G14" s="17" t="s">
+      <c r="G14" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="H14" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I14" s="12"/>
+      <c r="H14" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="10"/>
     </row>
     <row r="15" spans="1:12">
-      <c r="A15" s="10">
+      <c r="A15" s="8">
         <v>9</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="10">
-        <v>1</v>
-      </c>
-      <c r="D15" s="9" t="s">
+      <c r="C15" s="8">
+        <v>1</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="G15" s="17" t="s">
+      <c r="G15" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="H15" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I15" s="12"/>
+      <c r="H15" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" s="10"/>
     </row>
     <row r="16" spans="1:12">
-      <c r="A16" s="10">
+      <c r="A16" s="8">
         <v>10</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="10">
-        <v>1</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="C16" s="8">
+        <v>1</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="G16" s="17" t="s">
+      <c r="G16" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="H16" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I16" s="12"/>
+      <c r="H16" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I16" s="10"/>
     </row>
     <row r="17" spans="1:13">
-      <c r="A17" s="10">
+      <c r="A17" s="8">
         <v>11</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="8">
         <v>3</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G17" s="17" t="s">
+      <c r="G17" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="H17" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I17" s="12"/>
+      <c r="H17" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="10"/>
     </row>
     <row r="18" spans="1:13">
-      <c r="A18" s="10">
+      <c r="A18" s="8">
         <v>12</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <v>4</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="G18" s="17" t="s">
+      <c r="G18" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="H18" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I18" s="12"/>
-      <c r="M18" s="8"/>
+      <c r="H18" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="10"/>
+      <c r="M18" s="6"/>
     </row>
     <row r="19" spans="1:13">
-      <c r="A19" s="10">
+      <c r="A19" s="8">
         <v>13</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="10">
-        <v>1</v>
-      </c>
-      <c r="D19" s="9" t="s">
+      <c r="C19" s="8">
+        <v>1</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="F19" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="G19" s="17" t="s">
+      <c r="G19" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="H19" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I19" s="12"/>
+      <c r="H19" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I19" s="10"/>
     </row>
     <row r="20" spans="1:13">
-      <c r="A20" s="10">
+      <c r="A20" s="8">
         <v>14</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="8">
         <v>3</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="G20" s="17" t="s">
+      <c r="G20" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="H20" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I20" s="12"/>
-    </row>
-    <row r="21" spans="1:13" ht="69">
-      <c r="A21" s="10">
+      <c r="H20" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="10"/>
+    </row>
+    <row r="21" spans="1:13" ht="71.25">
+      <c r="A21" s="8">
         <v>15</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="8">
         <v>15</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="F21" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="G21" s="17" t="s">
+      <c r="G21" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="H21" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I21" s="12"/>
+      <c r="H21" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I21" s="10"/>
     </row>
     <row r="22" spans="1:13">
-      <c r="A22" s="10">
+      <c r="A22" s="8">
         <v>16</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="10">
+      <c r="C22" s="8">
         <v>2</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="G22" s="17" t="s">
+      <c r="G22" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="H22" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I22" s="12"/>
+      <c r="H22" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I22" s="10"/>
     </row>
     <row r="23" spans="1:13">
-      <c r="A23" s="10">
+      <c r="A23" s="8">
         <v>17</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="10">
-        <v>1</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="C23" s="8">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G23" s="17" t="s">
+      <c r="G23" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="H23" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I23" s="12"/>
+      <c r="H23" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I23" s="10"/>
     </row>
     <row r="24" spans="1:13">
-      <c r="A24" s="10">
+      <c r="A24" s="8">
         <v>18</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="8">
         <v>3</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G24" s="17" t="s">
+      <c r="G24" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="H24" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I24" s="12"/>
+      <c r="H24" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" s="10"/>
     </row>
     <row r="25" spans="1:13">
-      <c r="A25" s="10">
+      <c r="A25" s="8">
         <v>19</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="10">
+      <c r="C25" s="8">
         <v>2</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G25" s="17" t="s">
+      <c r="G25" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="H25" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I25" s="12"/>
-    </row>
-    <row r="26" spans="1:13" s="2" customFormat="1" ht="14.4">
-      <c r="A26" s="10">
+      <c r="H25" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I25" s="10"/>
+    </row>
+    <row r="26" spans="1:13" s="2" customFormat="1">
+      <c r="A26" s="8">
         <v>19</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="8">
         <v>2</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="G26" s="17" t="s">
+      <c r="G26" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="H26" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I26" s="12"/>
+      <c r="H26" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I26" s="10"/>
     </row>
     <row r="27" spans="1:13">
-      <c r="A27" s="10">
+      <c r="A27" s="8">
         <v>20</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="10">
-        <v>1</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="C27" s="8">
+        <v>1</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G27" s="17" t="s">
+      <c r="G27" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="H27" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I27" s="12"/>
+      <c r="H27" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" s="10"/>
     </row>
     <row r="28" spans="1:13">
-      <c r="A28" s="13">
+      <c r="A28" s="11">
         <v>21</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="C28" s="13">
-        <v>1</v>
-      </c>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="14" t="s">
+      <c r="C28" s="11">
+        <v>1</v>
+      </c>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G28" s="19"/>
+      <c r="H28" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="I28" s="10"/>
+    </row>
+    <row r="29" spans="1:13">
+      <c r="A29" s="8">
+        <v>22</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="8">
+        <v>1</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="H29" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="10"/>
+    </row>
+    <row r="30" spans="1:13">
+      <c r="A30" s="11">
+        <v>23</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="11">
+        <v>1</v>
+      </c>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="G30" s="19"/>
+      <c r="H30" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="I30" s="10"/>
+    </row>
+    <row r="31" spans="1:13">
+      <c r="A31" s="11">
+        <v>24</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C31" s="11">
+        <v>1</v>
+      </c>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="G31" s="19"/>
+      <c r="H31" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="I31" s="10"/>
+    </row>
+    <row r="32" spans="1:13">
+      <c r="A32" s="11">
+        <v>25</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" s="11">
+        <v>1</v>
+      </c>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="G32" s="19"/>
+      <c r="H32" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="I32" s="10"/>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="8">
+        <v>26</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C33" s="8">
+        <v>1</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="G28" s="21"/>
-      <c r="H28" s="15" t="s">
+      <c r="E33" s="17" t="s">
+        <v>115</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G33" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I33" s="10"/>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="20">
+        <v>27</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C34" s="8">
+        <v>1</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="G34" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I34" s="10"/>
+    </row>
+    <row r="35" spans="1:9" ht="28.5">
+      <c r="A35" s="20">
+        <v>28</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C35" s="8">
+        <v>5</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I35" s="10"/>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="20">
+        <v>29</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="C36" s="8">
+        <v>2</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I36" s="10"/>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="20">
+        <v>30</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C37" s="8">
+        <v>1</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="G37" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="I37" s="10"/>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="11">
+        <v>31</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C38" s="11">
+        <v>1</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="G38" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="H38" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="I28" s="12"/>
-    </row>
-    <row r="29" spans="1:13">
-      <c r="A29" s="10">
-        <v>22</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C29" s="10">
-        <v>1</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="G29" s="17" t="s">
-        <v>113</v>
-      </c>
-      <c r="H29" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="12"/>
-    </row>
-    <row r="30" spans="1:13">
-      <c r="A30" s="13">
-        <v>23</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C30" s="13">
-        <v>1</v>
-      </c>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="G30" s="21"/>
-      <c r="H30" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="I30" s="12"/>
-    </row>
-    <row r="31" spans="1:13">
-      <c r="A31" s="13">
-        <v>24</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="C31" s="13">
-        <v>1</v>
-      </c>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="G31" s="21"/>
-      <c r="H31" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="I31" s="12"/>
-    </row>
-    <row r="32" spans="1:13">
-      <c r="A32" s="13">
-        <v>25</v>
-      </c>
-      <c r="B32" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="C32" s="13">
-        <v>1</v>
-      </c>
-      <c r="D32" s="20"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="G32" s="21"/>
-      <c r="H32" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="I32" s="12"/>
-    </row>
-    <row r="33" spans="1:9">
-      <c r="A33" s="10">
-        <v>26</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C33" s="10">
-        <v>1</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="E33" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="F33" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="G33" s="17" t="s">
-        <v>118</v>
-      </c>
-      <c r="H33" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I33" s="12"/>
-    </row>
-    <row r="34" spans="1:9">
-      <c r="A34" s="22">
-        <v>27</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="C34" s="10">
-        <v>1</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="G34" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="H34" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I34" s="12"/>
-    </row>
-    <row r="35" spans="1:9" ht="27.6">
-      <c r="A35" s="22">
-        <v>28</v>
-      </c>
-      <c r="B35" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="C35" s="10">
-        <v>5</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="G35" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="H35" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I35" s="12"/>
-    </row>
-    <row r="36" spans="1:9">
-      <c r="A36" s="22">
-        <v>29</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="C36" s="10">
-        <v>2</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="G36" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="H36" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I36" s="12"/>
-    </row>
-    <row r="37" spans="1:9">
-      <c r="A37" s="22">
-        <v>30</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="C37" s="10">
-        <v>1</v>
-      </c>
-      <c r="D37" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="G37" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="H37" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I37" s="12"/>
-    </row>
-    <row r="38" spans="1:9">
-      <c r="A38" s="13">
-        <v>31</v>
-      </c>
-      <c r="B38" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="C38" s="13">
-        <v>1</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="F38" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="G38" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="H38" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="I38" s="12"/>
+      <c r="I38" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>